<commit_message>
Update MLB weather 2026-07-28 08:59 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v5_2026_07_29.xlsx
+++ b/mlb_weather_professional_v5_2026_07_29.xlsx
@@ -632,52 +632,52 @@
     <t>MEDIUM</t>
   </si>
   <si>
-    <t>2026-07-28 08:54:33 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:54:34 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:54:36 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:54:37 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:54:38 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:54:39 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:54:40 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:54:41 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:54:42 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:54:43 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:54:45 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:54:46 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:54:47 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:54:48 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:54:50 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:54:51 PM PDT</t>
+    <t>2026-07-28 08:58:49 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 08:58:50 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 08:58:51 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 08:58:53 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 08:58:54 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 08:58:55 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 08:58:56 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 08:58:57 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 08:58:58 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 08:58:59 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 08:59:00 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 08:59:01 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 08:59:02 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 08:59:03 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 08:59:04 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 08:59:05 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -1085,52 +1085,52 @@
     <t>10:10 PM PDT</t>
   </si>
   <si>
-    <t>2026-07-29 03:54:33 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:54:34 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:54:36 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:54:37 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:54:38 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:54:39 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:54:40 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:54:41 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:54:42 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:54:43 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:54:45 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:54:46 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:54:47 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:54:48 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:54:50 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:54:51 UTC</t>
+    <t>2026-07-29 03:58:49 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 03:58:50 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 03:58:51 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 03:58:53 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 03:58:54 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 03:58:55 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 03:58:56 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 03:58:57 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 03:58:58 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 03:58:59 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 03:59:00 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 03:59:01 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 03:59:02 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 03:59:03 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 03:59:04 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 03:59:05 UTC</t>
   </si>
   <si>
     <t>2026-07-28T20:31:41+00:00</t>
@@ -2074,7 +2074,7 @@
         <v>203</v>
       </c>
       <c r="AZ2">
-        <v>442.9</v>
+        <v>447.1</v>
       </c>
       <c r="BA2">
         <v>5</v>
@@ -2208,7 +2208,7 @@
         <v>194</v>
       </c>
       <c r="AR3">
-        <v>10.5</v>
+        <v>10.3</v>
       </c>
       <c r="AS3">
         <v>0</v>
@@ -2232,7 +2232,7 @@
         <v>204</v>
       </c>
       <c r="AZ3">
-        <v>347.9</v>
+        <v>352.2</v>
       </c>
       <c r="BA3">
         <v>5</v>
@@ -2366,7 +2366,7 @@
         <v>195</v>
       </c>
       <c r="AR4">
-        <v>-5.6</v>
+        <v>-5.3</v>
       </c>
       <c r="AS4">
         <v>0</v>
@@ -2390,7 +2390,7 @@
         <v>205</v>
       </c>
       <c r="AZ4">
-        <v>61.3</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="BA4">
         <v>5</v>
@@ -2479,7 +2479,7 @@
         <v>5.3</v>
       </c>
       <c r="AC5">
-        <v>91.2</v>
+        <v>91.3</v>
       </c>
       <c r="AD5" t="s">
         <v>192</v>
@@ -2524,7 +2524,7 @@
         <v>194</v>
       </c>
       <c r="AR5">
-        <v>9.6</v>
+        <v>9.9</v>
       </c>
       <c r="AS5">
         <v>0</v>
@@ -2548,7 +2548,7 @@
         <v>206</v>
       </c>
       <c r="AZ5">
-        <v>105.7</v>
+        <v>109.9</v>
       </c>
       <c r="BA5">
         <v>5</v>
@@ -2706,7 +2706,7 @@
         <v>207</v>
       </c>
       <c r="AZ6">
-        <v>152.9</v>
+        <v>157.2</v>
       </c>
       <c r="BA6">
         <v>5</v>
@@ -2840,7 +2840,7 @@
         <v>194</v>
       </c>
       <c r="AR7">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="AS7">
         <v>0</v>
@@ -2864,7 +2864,7 @@
         <v>208</v>
       </c>
       <c r="AZ7">
-        <v>448.2</v>
+        <v>452.5</v>
       </c>
       <c r="BA7">
         <v>5</v>
@@ -3022,7 +3022,7 @@
         <v>209</v>
       </c>
       <c r="AZ8">
-        <v>465.1</v>
+        <v>469.4</v>
       </c>
       <c r="BA8">
         <v>5</v>
@@ -3090,7 +3090,7 @@
         <v>172</v>
       </c>
       <c r="V9">
-        <v>26.1</v>
+        <v>26.4</v>
       </c>
       <c r="W9">
         <v>50</v>
@@ -3111,7 +3111,7 @@
         <v>0</v>
       </c>
       <c r="AC9">
-        <v>84.09999999999999</v>
+        <v>84.2</v>
       </c>
       <c r="AD9" t="s">
         <v>191</v>
@@ -3180,7 +3180,7 @@
         <v>210</v>
       </c>
       <c r="AZ9">
-        <v>533.7</v>
+        <v>538</v>
       </c>
       <c r="BA9">
         <v>5</v>
@@ -3314,7 +3314,7 @@
         <v>197</v>
       </c>
       <c r="AR10">
-        <v>-2.3</v>
+        <v>-2.4</v>
       </c>
       <c r="AS10">
         <v>0</v>
@@ -3338,7 +3338,7 @@
         <v>211</v>
       </c>
       <c r="AZ10">
-        <v>153</v>
+        <v>157.2</v>
       </c>
       <c r="BA10">
         <v>5</v>
@@ -3496,7 +3496,7 @@
         <v>212</v>
       </c>
       <c r="AZ11">
-        <v>474.1</v>
+        <v>478.4</v>
       </c>
       <c r="BA11">
         <v>5</v>
@@ -3654,7 +3654,7 @@
         <v>213</v>
       </c>
       <c r="AZ12">
-        <v>183.8</v>
+        <v>188</v>
       </c>
       <c r="BA12">
         <v>5</v>
@@ -3812,7 +3812,7 @@
         <v>214</v>
       </c>
       <c r="AZ13">
-        <v>93.40000000000001</v>
+        <v>97.7</v>
       </c>
       <c r="BA13">
         <v>5</v>
@@ -3946,7 +3946,7 @@
         <v>195</v>
       </c>
       <c r="AR14">
-        <v>-7.7</v>
+        <v>-7.9</v>
       </c>
       <c r="AS14">
         <v>0</v>
@@ -3970,7 +3970,7 @@
         <v>215</v>
       </c>
       <c r="AZ14">
-        <v>23.3</v>
+        <v>27.6</v>
       </c>
       <c r="BA14">
         <v>5</v>
@@ -4128,7 +4128,7 @@
         <v>216</v>
       </c>
       <c r="AZ15">
-        <v>465.2</v>
+        <v>469.5</v>
       </c>
       <c r="BA15">
         <v>5</v>
@@ -4286,7 +4286,7 @@
         <v>217</v>
       </c>
       <c r="AZ16">
-        <v>413.8</v>
+        <v>418</v>
       </c>
       <c r="BA16">
         <v>5</v>
@@ -4417,10 +4417,10 @@
         <v>67.59999999999999</v>
       </c>
       <c r="AQ17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AR17">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="AS17">
         <v>0</v>
@@ -4444,7 +4444,7 @@
         <v>218</v>
       </c>
       <c r="AZ17">
-        <v>33.2</v>
+        <v>37.4</v>
       </c>
       <c r="BA17">
         <v>5</v>
@@ -4914,10 +4914,10 @@
         <v>370</v>
       </c>
       <c r="J2">
-        <v>442.9</v>
+        <v>447.1</v>
       </c>
       <c r="K2">
-        <v>12.3</v>
+        <v>12.2</v>
       </c>
       <c r="L2">
         <v>5</v>
@@ -4959,7 +4959,7 @@
         <v>11.2</v>
       </c>
       <c r="Y2">
-        <v>90.8</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="Z2">
         <v>52.9</v>
@@ -5228,10 +5228,10 @@
         <v>370</v>
       </c>
       <c r="J3">
-        <v>442.9</v>
+        <v>447.1</v>
       </c>
       <c r="K3">
-        <v>13.3</v>
+        <v>13.2</v>
       </c>
       <c r="L3">
         <v>5</v>
@@ -5542,10 +5542,10 @@
         <v>370</v>
       </c>
       <c r="J4">
-        <v>442.9</v>
+        <v>447.1</v>
       </c>
       <c r="K4">
-        <v>14.3</v>
+        <v>14.2</v>
       </c>
       <c r="L4">
         <v>5</v>
@@ -5856,10 +5856,10 @@
         <v>370</v>
       </c>
       <c r="J5">
-        <v>442.9</v>
+        <v>447.1</v>
       </c>
       <c r="K5">
-        <v>15.3</v>
+        <v>15.2</v>
       </c>
       <c r="L5">
         <v>5</v>
@@ -6170,10 +6170,10 @@
         <v>371</v>
       </c>
       <c r="J6">
-        <v>347.9</v>
+        <v>352.2</v>
       </c>
       <c r="K6">
-        <v>12.7</v>
+        <v>12.6</v>
       </c>
       <c r="L6">
         <v>5</v>
@@ -6484,10 +6484,10 @@
         <v>371</v>
       </c>
       <c r="J7">
-        <v>347.9</v>
+        <v>352.2</v>
       </c>
       <c r="K7">
-        <v>13.7</v>
+        <v>13.6</v>
       </c>
       <c r="L7">
         <v>5</v>
@@ -6798,10 +6798,10 @@
         <v>371</v>
       </c>
       <c r="J8">
-        <v>347.9</v>
+        <v>352.2</v>
       </c>
       <c r="K8">
-        <v>14.7</v>
+        <v>14.6</v>
       </c>
       <c r="L8">
         <v>5</v>
@@ -7112,10 +7112,10 @@
         <v>371</v>
       </c>
       <c r="J9">
-        <v>347.9</v>
+        <v>352.2</v>
       </c>
       <c r="K9">
-        <v>15.7</v>
+        <v>15.6</v>
       </c>
       <c r="L9">
         <v>5</v>
@@ -7379,7 +7379,7 @@
         <v>200</v>
       </c>
       <c r="CU9">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="CV9" t="s">
         <v>200</v>
@@ -7426,10 +7426,10 @@
         <v>372</v>
       </c>
       <c r="J10">
-        <v>61.3</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="K10">
-        <v>13.2</v>
+        <v>13.1</v>
       </c>
       <c r="L10">
         <v>5</v>
@@ -7740,10 +7740,10 @@
         <v>372</v>
       </c>
       <c r="J11">
-        <v>61.3</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="K11">
-        <v>14.2</v>
+        <v>14.1</v>
       </c>
       <c r="L11">
         <v>5</v>
@@ -8054,10 +8054,10 @@
         <v>372</v>
       </c>
       <c r="J12">
-        <v>61.3</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="K12">
-        <v>15.2</v>
+        <v>15.1</v>
       </c>
       <c r="L12">
         <v>5</v>
@@ -8368,10 +8368,10 @@
         <v>372</v>
       </c>
       <c r="J13">
-        <v>61.3</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="K13">
-        <v>16.2</v>
+        <v>16.1</v>
       </c>
       <c r="L13">
         <v>5</v>
@@ -8682,10 +8682,10 @@
         <v>373</v>
       </c>
       <c r="J14">
-        <v>105.7</v>
+        <v>109.9</v>
       </c>
       <c r="K14">
-        <v>13.3</v>
+        <v>13.2</v>
       </c>
       <c r="L14">
         <v>5</v>
@@ -8727,7 +8727,7 @@
         <v>11.1</v>
       </c>
       <c r="Y14">
-        <v>92.09999999999999</v>
+        <v>92.2</v>
       </c>
       <c r="Z14">
         <v>78</v>
@@ -8996,10 +8996,10 @@
         <v>373</v>
       </c>
       <c r="J15">
-        <v>105.7</v>
+        <v>109.9</v>
       </c>
       <c r="K15">
-        <v>14.3</v>
+        <v>14.2</v>
       </c>
       <c r="L15">
         <v>5</v>
@@ -9310,10 +9310,10 @@
         <v>373</v>
       </c>
       <c r="J16">
-        <v>105.7</v>
+        <v>109.9</v>
       </c>
       <c r="K16">
-        <v>15.3</v>
+        <v>15.2</v>
       </c>
       <c r="L16">
         <v>5</v>
@@ -9624,10 +9624,10 @@
         <v>373</v>
       </c>
       <c r="J17">
-        <v>105.7</v>
+        <v>109.9</v>
       </c>
       <c r="K17">
-        <v>16.3</v>
+        <v>16.2</v>
       </c>
       <c r="L17">
         <v>5</v>
@@ -9938,10 +9938,10 @@
         <v>374</v>
       </c>
       <c r="J18">
-        <v>152.9</v>
+        <v>157.2</v>
       </c>
       <c r="K18">
-        <v>13.3</v>
+        <v>13.2</v>
       </c>
       <c r="L18">
         <v>5</v>
@@ -10252,10 +10252,10 @@
         <v>374</v>
       </c>
       <c r="J19">
-        <v>152.9</v>
+        <v>157.2</v>
       </c>
       <c r="K19">
-        <v>14.3</v>
+        <v>14.2</v>
       </c>
       <c r="L19">
         <v>5</v>
@@ -10566,10 +10566,10 @@
         <v>374</v>
       </c>
       <c r="J20">
-        <v>152.9</v>
+        <v>157.2</v>
       </c>
       <c r="K20">
-        <v>15.3</v>
+        <v>15.2</v>
       </c>
       <c r="L20">
         <v>5</v>
@@ -10880,10 +10880,10 @@
         <v>374</v>
       </c>
       <c r="J21">
-        <v>152.9</v>
+        <v>157.2</v>
       </c>
       <c r="K21">
-        <v>16.3</v>
+        <v>16.2</v>
       </c>
       <c r="L21">
         <v>5</v>
@@ -11194,7 +11194,7 @@
         <v>375</v>
       </c>
       <c r="J22">
-        <v>448.2</v>
+        <v>452.5</v>
       </c>
       <c r="K22">
         <v>15.8</v>
@@ -11508,7 +11508,7 @@
         <v>375</v>
       </c>
       <c r="J23">
-        <v>448.2</v>
+        <v>452.5</v>
       </c>
       <c r="K23">
         <v>16.8</v>
@@ -11822,7 +11822,7 @@
         <v>375</v>
       </c>
       <c r="J24">
-        <v>448.2</v>
+        <v>452.5</v>
       </c>
       <c r="K24">
         <v>17.8</v>
@@ -12136,7 +12136,7 @@
         <v>375</v>
       </c>
       <c r="J25">
-        <v>448.2</v>
+        <v>452.5</v>
       </c>
       <c r="K25">
         <v>18.8</v>
@@ -12450,10 +12450,10 @@
         <v>376</v>
       </c>
       <c r="J26">
-        <v>465.1</v>
+        <v>469.4</v>
       </c>
       <c r="K26">
-        <v>16.3</v>
+        <v>16.2</v>
       </c>
       <c r="L26">
         <v>5</v>
@@ -12764,10 +12764,10 @@
         <v>376</v>
       </c>
       <c r="J27">
-        <v>465.1</v>
+        <v>469.4</v>
       </c>
       <c r="K27">
-        <v>17.3</v>
+        <v>17.2</v>
       </c>
       <c r="L27">
         <v>5</v>
@@ -13078,10 +13078,10 @@
         <v>376</v>
       </c>
       <c r="J28">
-        <v>465.1</v>
+        <v>469.4</v>
       </c>
       <c r="K28">
-        <v>18.3</v>
+        <v>18.2</v>
       </c>
       <c r="L28">
         <v>5</v>
@@ -13392,10 +13392,10 @@
         <v>376</v>
       </c>
       <c r="J29">
-        <v>465.1</v>
+        <v>469.4</v>
       </c>
       <c r="K29">
-        <v>19.3</v>
+        <v>19.2</v>
       </c>
       <c r="L29">
         <v>5</v>
@@ -13706,10 +13706,10 @@
         <v>377</v>
       </c>
       <c r="J30">
-        <v>533.7</v>
+        <v>538</v>
       </c>
       <c r="K30">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="L30">
         <v>5</v>
@@ -13721,7 +13721,7 @@
         <v>2.27</v>
       </c>
       <c r="O30">
-        <v>12.92</v>
+        <v>12.42</v>
       </c>
       <c r="P30">
         <v>10.4</v>
@@ -13748,10 +13748,10 @@
         <v>0.6667</v>
       </c>
       <c r="X30">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="Y30">
-        <v>80.3</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="Z30">
         <v>52.7</v>
@@ -13793,7 +13793,7 @@
         <v>87</v>
       </c>
       <c r="AM30">
-        <v>26.1</v>
+        <v>26.4</v>
       </c>
       <c r="AN30">
         <v>0.001</v>
@@ -14020,10 +14020,10 @@
         <v>377</v>
       </c>
       <c r="J31">
-        <v>533.7</v>
+        <v>538</v>
       </c>
       <c r="K31">
-        <v>19.8</v>
+        <v>19.7</v>
       </c>
       <c r="L31">
         <v>5</v>
@@ -14334,10 +14334,10 @@
         <v>377</v>
       </c>
       <c r="J32">
-        <v>533.7</v>
+        <v>538</v>
       </c>
       <c r="K32">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
       <c r="L32">
         <v>5</v>
@@ -14648,10 +14648,10 @@
         <v>377</v>
       </c>
       <c r="J33">
-        <v>533.7</v>
+        <v>538</v>
       </c>
       <c r="K33">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
       <c r="L33">
         <v>5</v>
@@ -14962,10 +14962,10 @@
         <v>374</v>
       </c>
       <c r="J34">
-        <v>153</v>
+        <v>157.2</v>
       </c>
       <c r="K34">
-        <v>19.3</v>
+        <v>19.2</v>
       </c>
       <c r="L34">
         <v>5</v>
@@ -15276,10 +15276,10 @@
         <v>374</v>
       </c>
       <c r="J35">
-        <v>153</v>
+        <v>157.2</v>
       </c>
       <c r="K35">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="L35">
         <v>5</v>
@@ -15590,10 +15590,10 @@
         <v>374</v>
       </c>
       <c r="J36">
-        <v>153</v>
+        <v>157.2</v>
       </c>
       <c r="K36">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
       <c r="L36">
         <v>5</v>
@@ -15904,10 +15904,10 @@
         <v>374</v>
       </c>
       <c r="J37">
-        <v>153</v>
+        <v>157.2</v>
       </c>
       <c r="K37">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="L37">
         <v>5</v>
@@ -16218,10 +16218,10 @@
         <v>378</v>
       </c>
       <c r="J38">
-        <v>474.1</v>
+        <v>478.4</v>
       </c>
       <c r="K38">
-        <v>19.3</v>
+        <v>19.2</v>
       </c>
       <c r="L38">
         <v>5</v>
@@ -16532,10 +16532,10 @@
         <v>378</v>
       </c>
       <c r="J39">
-        <v>474.1</v>
+        <v>478.4</v>
       </c>
       <c r="K39">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="L39">
         <v>5</v>
@@ -16846,10 +16846,10 @@
         <v>378</v>
       </c>
       <c r="J40">
-        <v>474.1</v>
+        <v>478.4</v>
       </c>
       <c r="K40">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
       <c r="L40">
         <v>5</v>
@@ -17160,10 +17160,10 @@
         <v>378</v>
       </c>
       <c r="J41">
-        <v>474.1</v>
+        <v>478.4</v>
       </c>
       <c r="K41">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="L41">
         <v>5</v>
@@ -17474,10 +17474,10 @@
         <v>379</v>
       </c>
       <c r="J42">
-        <v>183.8</v>
+        <v>188</v>
       </c>
       <c r="K42">
-        <v>19.8</v>
+        <v>19.7</v>
       </c>
       <c r="L42">
         <v>5</v>
@@ -17788,10 +17788,10 @@
         <v>379</v>
       </c>
       <c r="J43">
-        <v>183.8</v>
+        <v>188</v>
       </c>
       <c r="K43">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
       <c r="L43">
         <v>5</v>
@@ -18055,7 +18055,7 @@
         <v>200</v>
       </c>
       <c r="CU43">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="CV43" t="s">
         <v>200</v>
@@ -18102,10 +18102,10 @@
         <v>379</v>
       </c>
       <c r="J44">
-        <v>183.8</v>
+        <v>188</v>
       </c>
       <c r="K44">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
       <c r="L44">
         <v>5</v>
@@ -18416,10 +18416,10 @@
         <v>379</v>
       </c>
       <c r="J45">
-        <v>183.8</v>
+        <v>188</v>
       </c>
       <c r="K45">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="L45">
         <v>5</v>
@@ -18730,10 +18730,10 @@
         <v>380</v>
       </c>
       <c r="J46">
-        <v>93.40000000000001</v>
+        <v>97.7</v>
       </c>
       <c r="K46">
-        <v>19.8</v>
+        <v>19.7</v>
       </c>
       <c r="L46">
         <v>5</v>
@@ -19044,10 +19044,10 @@
         <v>380</v>
       </c>
       <c r="J47">
-        <v>93.40000000000001</v>
+        <v>97.7</v>
       </c>
       <c r="K47">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
       <c r="L47">
         <v>5</v>
@@ -19358,10 +19358,10 @@
         <v>380</v>
       </c>
       <c r="J48">
-        <v>93.40000000000001</v>
+        <v>97.7</v>
       </c>
       <c r="K48">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
       <c r="L48">
         <v>5</v>
@@ -19672,10 +19672,10 @@
         <v>380</v>
       </c>
       <c r="J49">
-        <v>93.40000000000001</v>
+        <v>97.7</v>
       </c>
       <c r="K49">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="L49">
         <v>5</v>
@@ -19986,7 +19986,7 @@
         <v>381</v>
       </c>
       <c r="J50">
-        <v>23.3</v>
+        <v>27.6</v>
       </c>
       <c r="K50">
         <v>19.8</v>
@@ -20300,7 +20300,7 @@
         <v>381</v>
       </c>
       <c r="J51">
-        <v>23.3</v>
+        <v>27.6</v>
       </c>
       <c r="K51">
         <v>20.8</v>
@@ -20614,7 +20614,7 @@
         <v>381</v>
       </c>
       <c r="J52">
-        <v>23.3</v>
+        <v>27.6</v>
       </c>
       <c r="K52">
         <v>21.8</v>
@@ -20928,7 +20928,7 @@
         <v>381</v>
       </c>
       <c r="J53">
-        <v>23.3</v>
+        <v>27.6</v>
       </c>
       <c r="K53">
         <v>22.8</v>
@@ -21242,10 +21242,10 @@
         <v>376</v>
       </c>
       <c r="J54">
-        <v>465.2</v>
+        <v>469.5</v>
       </c>
       <c r="K54">
-        <v>21.7</v>
+        <v>21.6</v>
       </c>
       <c r="L54">
         <v>5</v>
@@ -21556,10 +21556,10 @@
         <v>376</v>
       </c>
       <c r="J55">
-        <v>465.2</v>
+        <v>469.5</v>
       </c>
       <c r="K55">
-        <v>22.7</v>
+        <v>22.6</v>
       </c>
       <c r="L55">
         <v>5</v>
@@ -21870,10 +21870,10 @@
         <v>376</v>
       </c>
       <c r="J56">
-        <v>465.2</v>
+        <v>469.5</v>
       </c>
       <c r="K56">
-        <v>23.7</v>
+        <v>23.6</v>
       </c>
       <c r="L56">
         <v>5</v>
@@ -22184,10 +22184,10 @@
         <v>376</v>
       </c>
       <c r="J57">
-        <v>465.2</v>
+        <v>469.5</v>
       </c>
       <c r="K57">
-        <v>24.7</v>
+        <v>24.6</v>
       </c>
       <c r="L57">
         <v>5</v>
@@ -22451,7 +22451,7 @@
         <v>200</v>
       </c>
       <c r="CU57">
-        <v>7.7</v>
+        <v>7.6</v>
       </c>
       <c r="CV57" t="s">
         <v>200</v>
@@ -22498,10 +22498,10 @@
         <v>382</v>
       </c>
       <c r="J58">
-        <v>413.8</v>
+        <v>418</v>
       </c>
       <c r="K58">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
       <c r="L58">
         <v>5</v>
@@ -22812,10 +22812,10 @@
         <v>382</v>
       </c>
       <c r="J59">
-        <v>413.8</v>
+        <v>418</v>
       </c>
       <c r="K59">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="L59">
         <v>5</v>
@@ -23126,10 +23126,10 @@
         <v>382</v>
       </c>
       <c r="J60">
-        <v>413.8</v>
+        <v>418</v>
       </c>
       <c r="K60">
-        <v>23.8</v>
+        <v>23.7</v>
       </c>
       <c r="L60">
         <v>5</v>
@@ -23393,7 +23393,7 @@
         <v>200</v>
       </c>
       <c r="CU60">
-        <v>5.1</v>
+        <v>5</v>
       </c>
       <c r="CV60" t="s">
         <v>200</v>
@@ -23440,10 +23440,10 @@
         <v>382</v>
       </c>
       <c r="J61">
-        <v>413.8</v>
+        <v>418</v>
       </c>
       <c r="K61">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="L61">
         <v>5</v>
@@ -23754,10 +23754,10 @@
         <v>383</v>
       </c>
       <c r="J62">
-        <v>33.2</v>
+        <v>37.4</v>
       </c>
       <c r="K62">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="L62">
         <v>5</v>
@@ -24068,10 +24068,10 @@
         <v>383</v>
       </c>
       <c r="J63">
-        <v>33.2</v>
+        <v>37.4</v>
       </c>
       <c r="K63">
-        <v>23.3</v>
+        <v>23.2</v>
       </c>
       <c r="L63">
         <v>5</v>
@@ -24382,10 +24382,10 @@
         <v>383</v>
       </c>
       <c r="J64">
-        <v>33.2</v>
+        <v>37.4</v>
       </c>
       <c r="K64">
-        <v>24.3</v>
+        <v>24.2</v>
       </c>
       <c r="L64">
         <v>5</v>
@@ -24696,10 +24696,10 @@
         <v>383</v>
       </c>
       <c r="J65">
-        <v>33.2</v>
+        <v>37.4</v>
       </c>
       <c r="K65">
-        <v>25.3</v>
+        <v>25.2</v>
       </c>
       <c r="L65">
         <v>5</v>
@@ -25139,7 +25139,7 @@
         <v>174</v>
       </c>
       <c r="G3">
-        <v>91.2</v>
+        <v>91.3</v>
       </c>
       <c r="H3">
         <v>11</v>
@@ -25881,7 +25881,7 @@
         <v>173</v>
       </c>
       <c r="G17">
-        <v>84.09999999999999</v>
+        <v>84.2</v>
       </c>
       <c r="H17">
         <v>0</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-28 09:01 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v5_2026_07_29.xlsx
+++ b/mlb_weather_professional_v5_2026_07_29.xlsx
@@ -632,52 +632,52 @@
     <t>MEDIUM</t>
   </si>
   <si>
-    <t>2026-07-28 08:58:49 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:58:50 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:58:51 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:58:53 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:58:54 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:58:55 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:58:56 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:58:57 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:58:58 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:58:59 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:59:00 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:59:01 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:59:02 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:59:03 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:59:04 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-28 08:59:05 PM PDT</t>
+    <t>2026-07-28 09:00:48 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 09:00:50 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 09:00:51 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 09:00:52 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 09:00:53 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 09:00:54 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 09:00:55 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 09:00:56 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 09:00:57 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 09:00:58 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 09:01:00 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 09:01:01 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 09:01:02 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 09:01:03 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 09:01:05 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-28 09:01:07 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -1085,52 +1085,52 @@
     <t>10:10 PM PDT</t>
   </si>
   <si>
-    <t>2026-07-29 03:58:49 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:58:50 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:58:51 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:58:53 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:58:54 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:58:55 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:58:56 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:58:57 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:58:58 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:58:59 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:59:00 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:59:01 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:59:02 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:59:03 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:59:04 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-29 03:59:05 UTC</t>
+    <t>2026-07-29 04:00:48 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 04:00:50 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 04:00:51 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 04:00:52 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 04:00:53 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 04:00:54 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 04:00:55 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 04:00:56 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 04:00:57 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 04:00:58 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 04:01:00 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 04:01:01 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 04:01:02 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 04:01:03 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 04:01:05 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-29 04:01:07 UTC</t>
   </si>
   <si>
     <t>2026-07-28T20:31:41+00:00</t>
@@ -1984,7 +1984,7 @@
         <v>172</v>
       </c>
       <c r="V2">
-        <v>13.9</v>
+        <v>13.8</v>
       </c>
       <c r="W2">
         <v>50</v>
@@ -2005,7 +2005,7 @@
         <v>0</v>
       </c>
       <c r="AC2">
-        <v>87.7</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="AD2" t="s">
         <v>191</v>
@@ -2074,7 +2074,7 @@
         <v>203</v>
       </c>
       <c r="AZ2">
-        <v>447.1</v>
+        <v>449.1</v>
       </c>
       <c r="BA2">
         <v>5</v>
@@ -2232,7 +2232,7 @@
         <v>204</v>
       </c>
       <c r="AZ3">
-        <v>352.2</v>
+        <v>354.2</v>
       </c>
       <c r="BA3">
         <v>5</v>
@@ -2390,7 +2390,7 @@
         <v>205</v>
       </c>
       <c r="AZ4">
-        <v>65.59999999999999</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="BA4">
         <v>5</v>
@@ -2548,7 +2548,7 @@
         <v>206</v>
       </c>
       <c r="AZ5">
-        <v>109.9</v>
+        <v>111.9</v>
       </c>
       <c r="BA5">
         <v>5</v>
@@ -2637,7 +2637,7 @@
         <v>1</v>
       </c>
       <c r="AC6">
-        <v>82.2</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="AD6" t="s">
         <v>191</v>
@@ -2694,7 +2694,7 @@
         <v>201</v>
       </c>
       <c r="AV6">
-        <v>37.4</v>
+        <v>37.2</v>
       </c>
       <c r="AW6" t="s">
         <v>200</v>
@@ -2706,7 +2706,7 @@
         <v>207</v>
       </c>
       <c r="AZ6">
-        <v>157.2</v>
+        <v>159.2</v>
       </c>
       <c r="BA6">
         <v>5</v>
@@ -2774,7 +2774,7 @@
         <v>172</v>
       </c>
       <c r="V7">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="W7">
         <v>55.3</v>
@@ -2864,7 +2864,7 @@
         <v>208</v>
       </c>
       <c r="AZ7">
-        <v>452.5</v>
+        <v>454.5</v>
       </c>
       <c r="BA7">
         <v>5</v>
@@ -3022,7 +3022,7 @@
         <v>209</v>
       </c>
       <c r="AZ8">
-        <v>469.4</v>
+        <v>471.4</v>
       </c>
       <c r="BA8">
         <v>5</v>
@@ -3180,7 +3180,7 @@
         <v>210</v>
       </c>
       <c r="AZ9">
-        <v>538</v>
+        <v>539.9</v>
       </c>
       <c r="BA9">
         <v>5</v>
@@ -3338,7 +3338,7 @@
         <v>211</v>
       </c>
       <c r="AZ10">
-        <v>157.2</v>
+        <v>159.2</v>
       </c>
       <c r="BA10">
         <v>5</v>
@@ -3496,7 +3496,7 @@
         <v>212</v>
       </c>
       <c r="AZ11">
-        <v>478.4</v>
+        <v>480.4</v>
       </c>
       <c r="BA11">
         <v>5</v>
@@ -3654,7 +3654,7 @@
         <v>213</v>
       </c>
       <c r="AZ12">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="BA12">
         <v>5</v>
@@ -3812,7 +3812,7 @@
         <v>214</v>
       </c>
       <c r="AZ13">
-        <v>97.7</v>
+        <v>99.7</v>
       </c>
       <c r="BA13">
         <v>5</v>
@@ -3970,7 +3970,7 @@
         <v>215</v>
       </c>
       <c r="AZ14">
-        <v>27.6</v>
+        <v>29.6</v>
       </c>
       <c r="BA14">
         <v>5</v>
@@ -4128,7 +4128,7 @@
         <v>216</v>
       </c>
       <c r="AZ15">
-        <v>469.5</v>
+        <v>471.5</v>
       </c>
       <c r="BA15">
         <v>5</v>
@@ -4286,7 +4286,7 @@
         <v>217</v>
       </c>
       <c r="AZ16">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="BA16">
         <v>5</v>
@@ -4444,7 +4444,7 @@
         <v>218</v>
       </c>
       <c r="AZ17">
-        <v>37.4</v>
+        <v>39.4</v>
       </c>
       <c r="BA17">
         <v>5</v>
@@ -4914,7 +4914,7 @@
         <v>370</v>
       </c>
       <c r="J2">
-        <v>447.1</v>
+        <v>449.1</v>
       </c>
       <c r="K2">
         <v>12.2</v>
@@ -4929,7 +4929,7 @@
         <v>0.62</v>
       </c>
       <c r="O2">
-        <v>13.82</v>
+        <v>13.91</v>
       </c>
       <c r="P2">
         <v>0.8</v>
@@ -4956,10 +4956,10 @@
         <v>0.1667</v>
       </c>
       <c r="X2">
-        <v>11.2</v>
+        <v>11.3</v>
       </c>
       <c r="Y2">
-        <v>90.90000000000001</v>
+        <v>90.8</v>
       </c>
       <c r="Z2">
         <v>52.9</v>
@@ -5001,7 +5001,7 @@
         <v>26.3</v>
       </c>
       <c r="AM2">
-        <v>13.9</v>
+        <v>13.8</v>
       </c>
       <c r="AN2">
         <v>0.002</v>
@@ -5228,7 +5228,7 @@
         <v>370</v>
       </c>
       <c r="J3">
-        <v>447.1</v>
+        <v>449.1</v>
       </c>
       <c r="K3">
         <v>13.2</v>
@@ -5243,7 +5243,7 @@
         <v>0.61</v>
       </c>
       <c r="O3">
-        <v>17.82</v>
+        <v>18.21</v>
       </c>
       <c r="P3">
         <v>4.2</v>
@@ -5270,10 +5270,10 @@
         <v>0.1667</v>
       </c>
       <c r="X3">
-        <v>14.1</v>
+        <v>14.2</v>
       </c>
       <c r="Y3">
-        <v>88.7</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="Z3">
         <v>52.8</v>
@@ -5315,7 +5315,7 @@
         <v>38.7</v>
       </c>
       <c r="AM3">
-        <v>19.4</v>
+        <v>19.1</v>
       </c>
       <c r="AN3">
         <v>0.002</v>
@@ -5542,7 +5542,7 @@
         <v>370</v>
       </c>
       <c r="J4">
-        <v>447.1</v>
+        <v>449.1</v>
       </c>
       <c r="K4">
         <v>14.2</v>
@@ -5557,7 +5557,7 @@
         <v>0.55</v>
       </c>
       <c r="O4">
-        <v>23.19</v>
+        <v>23.26</v>
       </c>
       <c r="P4">
         <v>9.699999999999999</v>
@@ -5856,7 +5856,7 @@
         <v>370</v>
       </c>
       <c r="J5">
-        <v>447.1</v>
+        <v>449.1</v>
       </c>
       <c r="K5">
         <v>15.2</v>
@@ -5871,7 +5871,7 @@
         <v>2.82</v>
       </c>
       <c r="O5">
-        <v>24.68</v>
+        <v>25</v>
       </c>
       <c r="P5">
         <v>36.5</v>
@@ -5898,10 +5898,10 @@
         <v>0.1667</v>
       </c>
       <c r="X5">
-        <v>34.1</v>
+        <v>34.2</v>
       </c>
       <c r="Y5">
-        <v>71.2</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="Z5">
         <v>52.3</v>
@@ -5943,7 +5943,7 @@
         <v>81.3</v>
       </c>
       <c r="AM5">
-        <v>25.7</v>
+        <v>25.5</v>
       </c>
       <c r="AN5">
         <v>0.004</v>
@@ -6170,7 +6170,7 @@
         <v>371</v>
       </c>
       <c r="J6">
-        <v>352.2</v>
+        <v>354.2</v>
       </c>
       <c r="K6">
         <v>12.6</v>
@@ -6484,7 +6484,7 @@
         <v>371</v>
       </c>
       <c r="J7">
-        <v>352.2</v>
+        <v>354.2</v>
       </c>
       <c r="K7">
         <v>13.6</v>
@@ -6798,7 +6798,7 @@
         <v>371</v>
       </c>
       <c r="J8">
-        <v>352.2</v>
+        <v>354.2</v>
       </c>
       <c r="K8">
         <v>14.6</v>
@@ -7112,7 +7112,7 @@
         <v>371</v>
       </c>
       <c r="J9">
-        <v>352.2</v>
+        <v>354.2</v>
       </c>
       <c r="K9">
         <v>15.6</v>
@@ -7426,7 +7426,7 @@
         <v>372</v>
       </c>
       <c r="J10">
-        <v>65.59999999999999</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="K10">
         <v>13.1</v>
@@ -7740,7 +7740,7 @@
         <v>372</v>
       </c>
       <c r="J11">
-        <v>65.59999999999999</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="K11">
         <v>14.1</v>
@@ -8054,7 +8054,7 @@
         <v>372</v>
       </c>
       <c r="J12">
-        <v>65.59999999999999</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="K12">
         <v>15.1</v>
@@ -8368,7 +8368,7 @@
         <v>372</v>
       </c>
       <c r="J13">
-        <v>65.59999999999999</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="K13">
         <v>16.1</v>
@@ -8682,7 +8682,7 @@
         <v>373</v>
       </c>
       <c r="J14">
-        <v>109.9</v>
+        <v>111.9</v>
       </c>
       <c r="K14">
         <v>13.2</v>
@@ -8996,7 +8996,7 @@
         <v>373</v>
       </c>
       <c r="J15">
-        <v>109.9</v>
+        <v>111.9</v>
       </c>
       <c r="K15">
         <v>14.2</v>
@@ -9310,7 +9310,7 @@
         <v>373</v>
       </c>
       <c r="J16">
-        <v>109.9</v>
+        <v>111.9</v>
       </c>
       <c r="K16">
         <v>15.2</v>
@@ -9624,7 +9624,7 @@
         <v>373</v>
       </c>
       <c r="J17">
-        <v>109.9</v>
+        <v>111.9</v>
       </c>
       <c r="K17">
         <v>16.2</v>
@@ -9938,7 +9938,7 @@
         <v>374</v>
       </c>
       <c r="J18">
-        <v>157.2</v>
+        <v>159.2</v>
       </c>
       <c r="K18">
         <v>13.2</v>
@@ -9953,7 +9953,7 @@
         <v>1.6</v>
       </c>
       <c r="O18">
-        <v>24.96</v>
+        <v>25.36</v>
       </c>
       <c r="P18">
         <v>14.6</v>
@@ -9980,10 +9980,10 @@
         <v>0.1667</v>
       </c>
       <c r="X18">
-        <v>26</v>
+        <v>26.1</v>
       </c>
       <c r="Y18">
-        <v>81.40000000000001</v>
+        <v>81.3</v>
       </c>
       <c r="Z18">
         <v>47.4</v>
@@ -10252,7 +10252,7 @@
         <v>374</v>
       </c>
       <c r="J19">
-        <v>157.2</v>
+        <v>159.2</v>
       </c>
       <c r="K19">
         <v>14.2</v>
@@ -10267,7 +10267,7 @@
         <v>1.21</v>
       </c>
       <c r="O19">
-        <v>25.75</v>
+        <v>25.9</v>
       </c>
       <c r="P19">
         <v>15.5</v>
@@ -10294,7 +10294,7 @@
         <v>0.1667</v>
       </c>
       <c r="X19">
-        <v>22.8</v>
+        <v>22.9</v>
       </c>
       <c r="Y19">
         <v>81.59999999999999</v>
@@ -10566,7 +10566,7 @@
         <v>374</v>
       </c>
       <c r="J20">
-        <v>157.2</v>
+        <v>159.2</v>
       </c>
       <c r="K20">
         <v>15.2</v>
@@ -10581,7 +10581,7 @@
         <v>1.28</v>
       </c>
       <c r="O20">
-        <v>25.46</v>
+        <v>26.2</v>
       </c>
       <c r="P20">
         <v>12.9</v>
@@ -10608,10 +10608,10 @@
         <v>0.1667</v>
       </c>
       <c r="X20">
-        <v>20.7</v>
+        <v>20.9</v>
       </c>
       <c r="Y20">
-        <v>83.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="Z20">
         <v>47.2</v>
@@ -10880,7 +10880,7 @@
         <v>374</v>
       </c>
       <c r="J21">
-        <v>157.2</v>
+        <v>159.2</v>
       </c>
       <c r="K21">
         <v>16.2</v>
@@ -10895,7 +10895,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="O21">
-        <v>27.48</v>
+        <v>27.93</v>
       </c>
       <c r="P21">
         <v>17.2</v>
@@ -10922,10 +10922,10 @@
         <v>0.1667</v>
       </c>
       <c r="X21">
-        <v>16.7</v>
+        <v>16.8</v>
       </c>
       <c r="Y21">
-        <v>84.3</v>
+        <v>84.2</v>
       </c>
       <c r="Z21">
         <v>46.9</v>
@@ -10967,7 +10967,7 @@
         <v>68.09999999999999</v>
       </c>
       <c r="AM21">
-        <v>43.6</v>
+        <v>43.2</v>
       </c>
       <c r="AN21">
         <v>0.004</v>
@@ -11141,7 +11141,7 @@
         <v>62.3</v>
       </c>
       <c r="CS21">
-        <v>37.4</v>
+        <v>37.2</v>
       </c>
       <c r="CT21" t="s">
         <v>201</v>
@@ -11194,10 +11194,10 @@
         <v>375</v>
       </c>
       <c r="J22">
-        <v>452.5</v>
+        <v>454.5</v>
       </c>
       <c r="K22">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="L22">
         <v>5</v>
@@ -11209,7 +11209,7 @@
         <v>3.01</v>
       </c>
       <c r="O22">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="P22">
         <v>11.2</v>
@@ -11281,7 +11281,7 @@
         <v>15</v>
       </c>
       <c r="AM22">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AN22">
         <v>0</v>
@@ -11508,10 +11508,10 @@
         <v>375</v>
       </c>
       <c r="J23">
-        <v>452.5</v>
+        <v>454.5</v>
       </c>
       <c r="K23">
-        <v>16.8</v>
+        <v>16.7</v>
       </c>
       <c r="L23">
         <v>5</v>
@@ -11822,10 +11822,10 @@
         <v>375</v>
       </c>
       <c r="J24">
-        <v>452.5</v>
+        <v>454.5</v>
       </c>
       <c r="K24">
-        <v>17.8</v>
+        <v>17.7</v>
       </c>
       <c r="L24">
         <v>5</v>
@@ -12136,10 +12136,10 @@
         <v>375</v>
       </c>
       <c r="J25">
-        <v>452.5</v>
+        <v>454.5</v>
       </c>
       <c r="K25">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="L25">
         <v>5</v>
@@ -12450,7 +12450,7 @@
         <v>376</v>
       </c>
       <c r="J26">
-        <v>469.4</v>
+        <v>471.4</v>
       </c>
       <c r="K26">
         <v>16.2</v>
@@ -12764,7 +12764,7 @@
         <v>376</v>
       </c>
       <c r="J27">
-        <v>469.4</v>
+        <v>471.4</v>
       </c>
       <c r="K27">
         <v>17.2</v>
@@ -13078,7 +13078,7 @@
         <v>376</v>
       </c>
       <c r="J28">
-        <v>469.4</v>
+        <v>471.4</v>
       </c>
       <c r="K28">
         <v>18.2</v>
@@ -13392,7 +13392,7 @@
         <v>376</v>
       </c>
       <c r="J29">
-        <v>469.4</v>
+        <v>471.4</v>
       </c>
       <c r="K29">
         <v>19.2</v>
@@ -13706,7 +13706,7 @@
         <v>377</v>
       </c>
       <c r="J30">
-        <v>538</v>
+        <v>539.9</v>
       </c>
       <c r="K30">
         <v>18.7</v>
@@ -14020,7 +14020,7 @@
         <v>377</v>
       </c>
       <c r="J31">
-        <v>538</v>
+        <v>539.9</v>
       </c>
       <c r="K31">
         <v>19.7</v>
@@ -14334,7 +14334,7 @@
         <v>377</v>
       </c>
       <c r="J32">
-        <v>538</v>
+        <v>539.9</v>
       </c>
       <c r="K32">
         <v>20.7</v>
@@ -14648,7 +14648,7 @@
         <v>377</v>
       </c>
       <c r="J33">
-        <v>538</v>
+        <v>539.9</v>
       </c>
       <c r="K33">
         <v>21.7</v>
@@ -14962,7 +14962,7 @@
         <v>374</v>
       </c>
       <c r="J34">
-        <v>157.2</v>
+        <v>159.2</v>
       </c>
       <c r="K34">
         <v>19.2</v>
@@ -15276,7 +15276,7 @@
         <v>374</v>
       </c>
       <c r="J35">
-        <v>157.2</v>
+        <v>159.2</v>
       </c>
       <c r="K35">
         <v>20.2</v>
@@ -15590,7 +15590,7 @@
         <v>374</v>
       </c>
       <c r="J36">
-        <v>157.2</v>
+        <v>159.2</v>
       </c>
       <c r="K36">
         <v>21.2</v>
@@ -15904,7 +15904,7 @@
         <v>374</v>
       </c>
       <c r="J37">
-        <v>157.2</v>
+        <v>159.2</v>
       </c>
       <c r="K37">
         <v>22.2</v>
@@ -16218,7 +16218,7 @@
         <v>378</v>
       </c>
       <c r="J38">
-        <v>478.4</v>
+        <v>480.4</v>
       </c>
       <c r="K38">
         <v>19.2</v>
@@ -16532,7 +16532,7 @@
         <v>378</v>
       </c>
       <c r="J39">
-        <v>478.4</v>
+        <v>480.4</v>
       </c>
       <c r="K39">
         <v>20.2</v>
@@ -16846,7 +16846,7 @@
         <v>378</v>
       </c>
       <c r="J40">
-        <v>478.4</v>
+        <v>480.4</v>
       </c>
       <c r="K40">
         <v>21.2</v>
@@ -17160,7 +17160,7 @@
         <v>378</v>
       </c>
       <c r="J41">
-        <v>478.4</v>
+        <v>480.4</v>
       </c>
       <c r="K41">
         <v>22.2</v>
@@ -17474,10 +17474,10 @@
         <v>379</v>
       </c>
       <c r="J42">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="K42">
-        <v>19.7</v>
+        <v>19.6</v>
       </c>
       <c r="L42">
         <v>5</v>
@@ -17788,10 +17788,10 @@
         <v>379</v>
       </c>
       <c r="J43">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="K43">
-        <v>20.7</v>
+        <v>20.6</v>
       </c>
       <c r="L43">
         <v>5</v>
@@ -18102,10 +18102,10 @@
         <v>379</v>
       </c>
       <c r="J44">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="K44">
-        <v>21.7</v>
+        <v>21.6</v>
       </c>
       <c r="L44">
         <v>5</v>
@@ -18416,10 +18416,10 @@
         <v>379</v>
       </c>
       <c r="J45">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="K45">
-        <v>22.7</v>
+        <v>22.6</v>
       </c>
       <c r="L45">
         <v>5</v>
@@ -18730,10 +18730,10 @@
         <v>380</v>
       </c>
       <c r="J46">
-        <v>97.7</v>
+        <v>99.7</v>
       </c>
       <c r="K46">
-        <v>19.7</v>
+        <v>19.6</v>
       </c>
       <c r="L46">
         <v>5</v>
@@ -19044,10 +19044,10 @@
         <v>380</v>
       </c>
       <c r="J47">
-        <v>97.7</v>
+        <v>99.7</v>
       </c>
       <c r="K47">
-        <v>20.7</v>
+        <v>20.6</v>
       </c>
       <c r="L47">
         <v>5</v>
@@ -19358,10 +19358,10 @@
         <v>380</v>
       </c>
       <c r="J48">
-        <v>97.7</v>
+        <v>99.7</v>
       </c>
       <c r="K48">
-        <v>21.7</v>
+        <v>21.6</v>
       </c>
       <c r="L48">
         <v>5</v>
@@ -19672,10 +19672,10 @@
         <v>380</v>
       </c>
       <c r="J49">
-        <v>97.7</v>
+        <v>99.7</v>
       </c>
       <c r="K49">
-        <v>22.7</v>
+        <v>22.6</v>
       </c>
       <c r="L49">
         <v>5</v>
@@ -19986,10 +19986,10 @@
         <v>381</v>
       </c>
       <c r="J50">
-        <v>27.6</v>
+        <v>29.6</v>
       </c>
       <c r="K50">
-        <v>19.8</v>
+        <v>19.7</v>
       </c>
       <c r="L50">
         <v>5</v>
@@ -20300,10 +20300,10 @@
         <v>381</v>
       </c>
       <c r="J51">
-        <v>27.6</v>
+        <v>29.6</v>
       </c>
       <c r="K51">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
       <c r="L51">
         <v>5</v>
@@ -20614,10 +20614,10 @@
         <v>381</v>
       </c>
       <c r="J52">
-        <v>27.6</v>
+        <v>29.6</v>
       </c>
       <c r="K52">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
       <c r="L52">
         <v>5</v>
@@ -20928,10 +20928,10 @@
         <v>381</v>
       </c>
       <c r="J53">
-        <v>27.6</v>
+        <v>29.6</v>
       </c>
       <c r="K53">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="L53">
         <v>5</v>
@@ -21242,7 +21242,7 @@
         <v>376</v>
       </c>
       <c r="J54">
-        <v>469.5</v>
+        <v>471.5</v>
       </c>
       <c r="K54">
         <v>21.6</v>
@@ -21556,7 +21556,7 @@
         <v>376</v>
       </c>
       <c r="J55">
-        <v>469.5</v>
+        <v>471.5</v>
       </c>
       <c r="K55">
         <v>22.6</v>
@@ -21870,7 +21870,7 @@
         <v>376</v>
       </c>
       <c r="J56">
-        <v>469.5</v>
+        <v>471.5</v>
       </c>
       <c r="K56">
         <v>23.6</v>
@@ -22184,7 +22184,7 @@
         <v>376</v>
       </c>
       <c r="J57">
-        <v>469.5</v>
+        <v>471.5</v>
       </c>
       <c r="K57">
         <v>24.6</v>
@@ -22498,10 +22498,10 @@
         <v>382</v>
       </c>
       <c r="J58">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="K58">
-        <v>21.7</v>
+        <v>21.6</v>
       </c>
       <c r="L58">
         <v>5</v>
@@ -22812,10 +22812,10 @@
         <v>382</v>
       </c>
       <c r="J59">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="K59">
-        <v>22.7</v>
+        <v>22.6</v>
       </c>
       <c r="L59">
         <v>5</v>
@@ -23126,10 +23126,10 @@
         <v>382</v>
       </c>
       <c r="J60">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="K60">
-        <v>23.7</v>
+        <v>23.6</v>
       </c>
       <c r="L60">
         <v>5</v>
@@ -23440,10 +23440,10 @@
         <v>382</v>
       </c>
       <c r="J61">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="K61">
-        <v>24.7</v>
+        <v>24.6</v>
       </c>
       <c r="L61">
         <v>5</v>
@@ -23754,10 +23754,10 @@
         <v>383</v>
       </c>
       <c r="J62">
-        <v>37.4</v>
+        <v>39.4</v>
       </c>
       <c r="K62">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="L62">
         <v>5</v>
@@ -24068,10 +24068,10 @@
         <v>383</v>
       </c>
       <c r="J63">
-        <v>37.4</v>
+        <v>39.4</v>
       </c>
       <c r="K63">
-        <v>23.2</v>
+        <v>23.1</v>
       </c>
       <c r="L63">
         <v>5</v>
@@ -24382,10 +24382,10 @@
         <v>383</v>
       </c>
       <c r="J64">
-        <v>37.4</v>
+        <v>39.4</v>
       </c>
       <c r="K64">
-        <v>24.2</v>
+        <v>24.1</v>
       </c>
       <c r="L64">
         <v>5</v>
@@ -24696,10 +24696,10 @@
         <v>383</v>
       </c>
       <c r="J65">
-        <v>37.4</v>
+        <v>39.4</v>
       </c>
       <c r="K65">
-        <v>25.2</v>
+        <v>25.1</v>
       </c>
       <c r="L65">
         <v>5</v>
@@ -25722,7 +25722,7 @@
         <v>173</v>
       </c>
       <c r="G14">
-        <v>82.2</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="H14">
         <v>2</v>
@@ -25828,7 +25828,7 @@
         <v>173</v>
       </c>
       <c r="G16">
-        <v>87.7</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="H16">
         <v>0</v>

</xml_diff>